<commit_message>
Complete Login module testing portfolio - add build 1.1
</commit_message>
<xml_diff>
--- a/09_Test_Execution/Build_1.1.xlsx
+++ b/09_Test_Execution/Build_1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Manual-Tester-Portfolio\09_Test_Execution\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81C8B6B6-344E-4EB2-86FD-F93AC8528D45}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8ABBC0C-E21E-41B9-AF9A-DBC2BDB15416}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8CF50AD5-48A9-485B-9342-A3CB8A421147}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="89">
   <si>
     <t>TC ID</t>
   </si>
@@ -73,9 +73,6 @@
   </si>
   <si>
     <t>Pass</t>
-  </si>
-  <si>
-    <t>Block</t>
   </si>
   <si>
     <t>TC_LOGIN_001</t>
@@ -266,12 +263,6 @@
   </si>
   <si>
     <t>Đăng nhập thất bại. Hiển thị thông báo "Email hoặc Password không đúng."</t>
-  </si>
-  <si>
-    <t>Không thể xác nhận chức năng mở khóa sau 15 phút vì tài khoản không bị khóa ở TC015.</t>
-  </si>
-  <si>
-    <t>Không thể kiểm tra chức năng Ẩn Password vì chức năng Show Password không hoạt động.</t>
   </si>
   <si>
     <t>Đăng nhập thành công khi không chọn Remember Me. Sau khi đóng trình duyệt, hệ thống yêu cầu đăng nhập lại.</t>
@@ -289,34 +280,32 @@
 Tài khoản chưa bị khóa.</t>
   </si>
   <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Critical</t>
-  </si>
-  <si>
-    <t>BUG_LOGIN_001</t>
-  </si>
-  <si>
-    <t>BUG_LOGIN_002</t>
-  </si>
-  <si>
-    <t>BUG_LOGIN_003</t>
-  </si>
-  <si>
-    <t>BUG_LOGIN_004</t>
-  </si>
-  <si>
-    <t>BUG_LOGIN_005</t>
-  </si>
-  <si>
-    <t>BUG_LOGIN_006</t>
-  </si>
-  <si>
     <t>Build 1.1</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công.
+Dashboard hiển thị "Xin chào Nguyễn Văn A".</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Password có 7 ký tự.</t>
+  </si>
+  <si>
+    <t>Không cho phép đăng nhập với Password có 21 ký tự.</t>
+  </si>
+  <si>
+    <t>Sau lần đăng nhập sai thứ 6, tài khoản bị khóa trong 15 phút.</t>
+  </si>
+  <si>
+    <t>Sau khi hết thời gian khóa 15 phút, người dùng đăng nhập thành công và chuyển đến Dashboard.</t>
+  </si>
+  <si>
+    <t>Nhấn lại biểu tượng Show Password, Password được ẩn bằng ký tự che.</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công. Hệ thống ghi nhớ trạng thái đăng nhập sau khi đóng và mở lại trình duyệt.</t>
+  </si>
+  <si>
+    <t>Sau khi đóng và mở lại trình duyệt, người dùng vẫn ở trạng thái đăng nhập.</t>
   </si>
 </sst>
 </file>
@@ -899,54 +888,51 @@
     </row>
     <row r="2" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
       <c r="F2" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H2" s="5"/>
+        <v>36</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>81</v>
+      </c>
       <c r="I2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="J2" s="3"/>
       <c r="L2" s="5"/>
     </row>
     <row r="3" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>12</v>
@@ -957,24 +943,24 @@
     </row>
     <row r="4" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
       <c r="F4" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>12</v>
@@ -985,24 +971,24 @@
     </row>
     <row r="5" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>12</v>
@@ -1013,24 +999,24 @@
     </row>
     <row r="6" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
       <c r="F6" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I6" s="3" t="s">
         <v>12</v>
@@ -1041,54 +1027,51 @@
     </row>
     <row r="7" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="H7" s="10"/>
+        <v>40</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>82</v>
+      </c>
       <c r="I7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>87</v>
-      </c>
+      <c r="J7" s="3"/>
       <c r="L7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
       <c r="F8" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>12</v>
@@ -1099,24 +1082,24 @@
     </row>
     <row r="9" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>12</v>
@@ -1127,54 +1110,51 @@
     </row>
     <row r="10" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="F10" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H10" s="5"/>
+        <v>42</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="I10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J10" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>88</v>
-      </c>
+      <c r="J10" s="3"/>
       <c r="L10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
       <c r="F11" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>12</v>
@@ -1185,24 +1165,24 @@
     </row>
     <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
       <c r="F12" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>12</v>
@@ -1213,24 +1193,24 @@
     </row>
     <row r="13" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
       <c r="F13" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>12</v>
@@ -1241,24 +1221,24 @@
     </row>
     <row r="14" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>12</v>
@@ -1269,24 +1249,24 @@
     </row>
     <row r="15" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
       <c r="F15" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>12</v>
@@ -1297,57 +1277,54 @@
     </row>
     <row r="16" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="H16" s="5"/>
+        <v>44</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>84</v>
+      </c>
       <c r="I16" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J16" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>89</v>
-      </c>
+      <c r="J16" s="3"/>
       <c r="L16" s="5"/>
     </row>
     <row r="17" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
@@ -1355,57 +1332,54 @@
     </row>
     <row r="18" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
       <c r="F18" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="H18" s="5"/>
+        <v>46</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="I18" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J18" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>90</v>
-      </c>
+      <c r="J18" s="3"/>
       <c r="L18" s="5"/>
     </row>
     <row r="19" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
@@ -1413,54 +1387,51 @@
     </row>
     <row r="20" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
       <c r="F20" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H20" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="I20" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J20" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="K20" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="J20" s="3"/>
       <c r="L20" s="5"/>
     </row>
     <row r="21" spans="1:12" ht="49.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
       <c r="F21" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>12</v>
@@ -1471,54 +1442,51 @@
     </row>
     <row r="22" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
       <c r="F22" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="H22" s="2"/>
+        <v>50</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="I22" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J22" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="K22" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="J22" s="3"/>
       <c r="L22" s="5"/>
     </row>
     <row r="23" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
       <c r="F23" s="7" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>12</v>

</xml_diff>